<commit_message>
Finishing touches on dashboard, finished PDM with stitched vias, continued work on dashboard teensy code
</commit_message>
<xml_diff>
--- a/PCB/DigitalDashDisplay2027/DigitalDashDisplay2027/JLCPCB Docs/BOM_Dash.xlsx
+++ b/PCB/DigitalDashDisplay2027/DigitalDashDisplay2027/JLCPCB Docs/BOM_Dash.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/DigitalDashDisplay2027/DigitalDashDisplay2027/JLCPCB Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{81882892-F37D-436E-9463-A799B2E805F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90EDC8B5-2E5E-4256-8471-4B2D4B8457C4}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{81882892-F37D-436E-9463-A799B2E805F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EC840B0-B3C4-4897-B67A-70633650C5E0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{640F1A2B-D9EF-4CC7-A694-2A33FF3CD11D}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
   <si>
     <t>Designator</t>
   </si>
@@ -89,12 +89,6 @@
     <t>LMR51430YDDCR</t>
   </si>
   <si>
-    <t>ILI1</t>
-  </si>
-  <si>
-    <t>ILI9488</t>
-  </si>
-  <si>
     <t>~</t>
   </si>
   <si>
@@ -122,12 +116,6 @@
     <t>ERJ-3EKF1372V</t>
   </si>
   <si>
-    <t>R3, R4</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
     <t>R5</t>
   </si>
   <si>
@@ -149,66 +137,18 @@
     <t>100k</t>
   </si>
   <si>
-    <t>R9, R10</t>
-  </si>
-  <si>
     <t>R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</t>
   </si>
   <si>
     <t>10k</t>
   </si>
   <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>R_1206_3216Metric</t>
-  </si>
-  <si>
-    <t>CSR1206FT50L0</t>
-  </si>
-  <si>
-    <t>REF**</t>
-  </si>
-  <si>
-    <t>Adafruit 254</t>
-  </si>
-  <si>
-    <t>T1</t>
-  </si>
-  <si>
-    <t>AC1210-110-C</t>
-  </si>
-  <si>
     <t>T2</t>
   </si>
   <si>
     <t>NCS2005SN1T1G</t>
   </si>
   <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>Teensy40_SMT</t>
-  </si>
-  <si>
-    <t>Teensy4.0</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>CONN08_533750810_MOL</t>
-  </si>
-  <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>U4</t>
-  </si>
-  <si>
-    <t>ESP32</t>
-  </si>
-  <si>
     <t>U5</t>
   </si>
   <si>
@@ -261,6 +201,12 @@
   </si>
   <si>
     <t>C15401</t>
+  </si>
+  <si>
+    <t>C5210749</t>
+  </si>
+  <si>
+    <t>R9, R10, R12</t>
   </si>
 </sst>
 </file>
@@ -632,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3643D93D-D7E1-48CE-99C1-35BDECE1D191}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
@@ -647,7 +593,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -656,7 +602,7 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -670,12 +616,12 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -684,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -698,7 +644,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -711,30 +657,36 @@
       <c r="C5" t="s">
         <v>11</v>
       </c>
+      <c r="D5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
+      <c r="D6" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>18</v>
       </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -742,38 +694,41 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
         <v>25</v>
       </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -781,13 +736,13 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -795,27 +750,27 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
         <v>29</v>
       </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
         <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -829,112 +784,7 @@
         <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>15</v>
-      </c>
-      <c r="B20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>